<commit_message>
check existing bso has same org as user selected org
</commit_message>
<xml_diff>
--- a/spec/fixtures/batch_submission_manifest_errors_parents.xlsx
+++ b/spec/fixtures/batch_submission_manifest_errors_parents.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10410"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smc101/vagrant/morphosource-vagrant/MorphoSource_SF/spec/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7C6C3BA-FA0B-D341-A72A-3C498C17E751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64CF0A10-C20A-BE46-886E-4B87F0F50073}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="283">
   <si>
     <t>Field Section</t>
   </si>
@@ -926,6 +926,15 @@
   </si>
   <si>
     <t>Geometry</t>
+  </si>
+  <si>
+    <t>ANSP_Fish_131736_Head.zip</t>
+  </si>
+  <si>
+    <t>Raw</t>
+  </si>
+  <si>
+    <t>TESTBSO123</t>
   </si>
 </sst>
 </file>
@@ -3442,8 +3451,206 @@
         <v>256</v>
       </c>
     </row>
-    <row r="11" spans="1:86" ht="16" x14ac:dyDescent="0.2">
-      <c r="BB11" s="49"/>
+    <row r="11" spans="1:86" ht="17" x14ac:dyDescent="0.2">
+      <c r="A11" s="32"/>
+      <c r="B11" s="32"/>
+      <c r="C11" s="49" t="s">
+        <v>280</v>
+      </c>
+      <c r="D11" s="40"/>
+      <c r="E11" s="28" t="s">
+        <v>235</v>
+      </c>
+      <c r="F11" s="49" t="s">
+        <v>281</v>
+      </c>
+      <c r="G11" s="34"/>
+      <c r="H11" s="42"/>
+      <c r="I11" s="33" t="s">
+        <v>282</v>
+      </c>
+      <c r="K11" s="28"/>
+      <c r="L11" s="28"/>
+      <c r="M11" s="34" t="s">
+        <v>266</v>
+      </c>
+      <c r="N11" s="34" t="s">
+        <v>267</v>
+      </c>
+      <c r="O11" s="28" t="s">
+        <v>236</v>
+      </c>
+      <c r="P11" s="28" t="s">
+        <v>237</v>
+      </c>
+      <c r="Q11" s="34" t="s">
+        <v>243</v>
+      </c>
+      <c r="R11" s="28" t="s">
+        <v>238</v>
+      </c>
+      <c r="S11" s="29"/>
+      <c r="T11" s="29"/>
+      <c r="U11" s="30"/>
+      <c r="V11" s="30"/>
+      <c r="W11" s="35">
+        <v>44177</v>
+      </c>
+      <c r="X11" s="30"/>
+      <c r="Y11" s="29">
+        <v>2.169024E-2</v>
+      </c>
+      <c r="Z11" s="29">
+        <v>2.169024E-2</v>
+      </c>
+      <c r="AA11" s="29">
+        <v>2.169024E-2</v>
+      </c>
+      <c r="AB11" s="29">
+        <v>8</v>
+      </c>
+      <c r="AC11" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="AD11" s="28" t="s">
+        <v>239</v>
+      </c>
+      <c r="AE11" s="34"/>
+      <c r="AF11" s="28"/>
+      <c r="AG11" s="28"/>
+      <c r="AH11" s="35">
+        <v>44177</v>
+      </c>
+      <c r="AI11" s="28"/>
+      <c r="AJ11" s="28"/>
+      <c r="AK11" s="28"/>
+      <c r="AL11" s="28"/>
+      <c r="AM11" s="28"/>
+      <c r="AN11" s="28"/>
+      <c r="AO11" s="28"/>
+      <c r="AP11" s="34" t="s">
+        <v>240</v>
+      </c>
+      <c r="AQ11" s="36" t="s">
+        <v>244</v>
+      </c>
+      <c r="AR11" s="28" t="s">
+        <v>240</v>
+      </c>
+      <c r="AS11" s="28" t="s">
+        <v>259</v>
+      </c>
+      <c r="AT11" s="28" t="s">
+        <v>260</v>
+      </c>
+      <c r="AU11" s="28"/>
+      <c r="AV11" s="34" t="s">
+        <v>248</v>
+      </c>
+      <c r="AW11" s="28" t="s">
+        <v>274</v>
+      </c>
+      <c r="AX11" s="38" t="s">
+        <v>249</v>
+      </c>
+      <c r="AY11" s="39">
+        <v>44502</v>
+      </c>
+      <c r="AZ11" s="29">
+        <v>0.200098</v>
+      </c>
+      <c r="BA11" s="28" t="s">
+        <v>241</v>
+      </c>
+      <c r="BB11" s="49" t="s">
+        <v>279</v>
+      </c>
+      <c r="BC11" s="28" t="s">
+        <v>240</v>
+      </c>
+      <c r="BD11">
+        <v>888</v>
+      </c>
+      <c r="BE11" s="29">
+        <v>3</v>
+      </c>
+      <c r="BF11" s="29">
+        <v>1680</v>
+      </c>
+      <c r="BG11" s="29">
+        <v>70</v>
+      </c>
+      <c r="BH11" s="29">
+        <v>1.4E-2</v>
+      </c>
+      <c r="BI11" s="29">
+        <v>200</v>
+      </c>
+      <c r="BJ11" s="34" t="s">
+        <v>252</v>
+      </c>
+      <c r="BK11" s="34" t="s">
+        <v>252</v>
+      </c>
+      <c r="BL11" s="34" t="s">
+        <v>250</v>
+      </c>
+      <c r="BM11" s="28" t="s">
+        <v>251</v>
+      </c>
+      <c r="BN11" s="28">
+        <v>90</v>
+      </c>
+      <c r="BO11">
+        <v>1</v>
+      </c>
+      <c r="BP11">
+        <v>1</v>
+      </c>
+      <c r="BQ11">
+        <v>1</v>
+      </c>
+      <c r="BR11" t="s">
+        <v>253</v>
+      </c>
+      <c r="BS11" t="s">
+        <v>252</v>
+      </c>
+      <c r="BT11" t="s">
+        <v>252</v>
+      </c>
+      <c r="BU11" t="s">
+        <v>252</v>
+      </c>
+      <c r="BV11">
+        <v>90</v>
+      </c>
+      <c r="BW11" t="s">
+        <v>240</v>
+      </c>
+      <c r="BX11" t="s">
+        <v>240</v>
+      </c>
+      <c r="BY11" s="28" t="s">
+        <v>254</v>
+      </c>
+      <c r="BZ11" s="34"/>
+      <c r="CA11" s="34"/>
+      <c r="CB11" s="34"/>
+      <c r="CC11" s="34"/>
+      <c r="CD11" s="34"/>
+      <c r="CE11" s="28" t="s">
+        <v>274</v>
+      </c>
+      <c r="CF11" s="35">
+        <v>44502</v>
+      </c>
+      <c r="CG11" s="34" t="s">
+        <v>255</v>
+      </c>
+      <c r="CH11" s="34" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="12" spans="1:86" ht="16" x14ac:dyDescent="0.2">
       <c r="BB12" s="49"/>

</xml_diff>